<commit_message>
Added fiberclamps, M05X, applied to TAboard
</commit_message>
<xml_diff>
--- a/Production/Pyopticl parts list.xlsx
+++ b/Production/Pyopticl parts list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kim/Desktop/Lab/Github/PyOpticL_Rubidium_System/Production/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF47C21-431D-DA41-97CC-6E1B30686599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2904F97F-50AD-A44E-B569-9DC9913C8B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14700" yWindow="740" windowWidth="14700" windowHeight="16680" xr2:uid="{2C0518BD-81B3-2E40-93F6-7012D65C5310}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16680" xr2:uid="{2C0518BD-81B3-2E40-93F6-7012D65C5310}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>